<commit_message>
feat(vtable): 增强 DDBaseGridVtable 支持自定义工具栏按钮 并接通 test0001 页面
</commit_message>
<xml_diff>
--- a/public/import_template/v0.2node/node_module.xlsx
+++ b/public/import_template/v0.2node/node_module.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\ddit\code\umi_max.260226_github\public\import_template\v0.2node\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0908BCD0-0D6F-41A6-AC17-9C2653A62522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DC96FE-4A21-4321-B201-D19F6DB3822A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="762" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="762" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="表" sheetId="8" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2334" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="748">
   <si>
     <t>字段中文名</t>
   </si>
@@ -2729,6 +2729,26 @@
   </si>
   <si>
     <t>./easy_dev_dc/example/dict_module_media_ns</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>./common/automatic_page_enh</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>进货明细E</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>/dynamicbs1/enh/cfgp/eg_m_mts_tsjh</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>出口明细E</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>/dynamicbs1/enh/cfgp/eg_m_mts_tssb</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2852,7 +2872,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2952,6 +2972,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3068,7 +3094,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3190,6 +3216,26 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3207,19 +3253,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6656,7 +6689,7 @@
       <c r="C205" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D205" s="52"/>
+      <c r="D205" s="46"/>
       <c r="E205" s="27"/>
       <c r="F205" s="27"/>
       <c r="G205" s="26"/>
@@ -6685,7 +6718,7 @@
       <c r="D207" s="26" t="s">
         <v>235</v>
       </c>
-      <c r="E207" s="52"/>
+      <c r="E207" s="46"/>
       <c r="F207" s="26" t="s">
         <v>236</v>
       </c>
@@ -6702,7 +6735,7 @@
         <v>455</v>
       </c>
       <c r="D208" s="26"/>
-      <c r="E208" s="52"/>
+      <c r="E208" s="46"/>
       <c r="F208" s="26"/>
       <c r="G208" s="26"/>
     </row>
@@ -6716,8 +6749,8 @@
       <c r="C209" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D209" s="52"/>
-      <c r="E209" s="52"/>
+      <c r="D209" s="46"/>
+      <c r="E209" s="46"/>
       <c r="F209" s="27"/>
       <c r="G209" s="26"/>
     </row>
@@ -8070,45 +8103,45 @@
       </c>
     </row>
     <row r="2" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="53" t="s">
         <v>533</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="46"/>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="46"/>
-      <c r="W2" s="46"/>
-      <c r="X2" s="46"/>
-      <c r="Y2" s="46"/>
-      <c r="Z2" s="46"/>
-      <c r="AA2" s="46"/>
-      <c r="AB2" s="46"/>
-      <c r="AC2" s="46"/>
-      <c r="AD2" s="46"/>
-      <c r="AE2" s="46"/>
-      <c r="AF2" s="46"/>
-      <c r="AG2" s="46"/>
-      <c r="AH2" s="46"/>
-      <c r="AI2" s="46"/>
-      <c r="AJ2" s="46"/>
-      <c r="AK2" s="47"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="54"/>
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+      <c r="Q2" s="54"/>
+      <c r="R2" s="54"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
+      <c r="V2" s="54"/>
+      <c r="W2" s="54"/>
+      <c r="X2" s="54"/>
+      <c r="Y2" s="54"/>
+      <c r="Z2" s="54"/>
+      <c r="AA2" s="54"/>
+      <c r="AB2" s="54"/>
+      <c r="AC2" s="54"/>
+      <c r="AD2" s="54"/>
+      <c r="AE2" s="54"/>
+      <c r="AF2" s="54"/>
+      <c r="AG2" s="54"/>
+      <c r="AH2" s="54"/>
+      <c r="AI2" s="54"/>
+      <c r="AJ2" s="54"/>
+      <c r="AK2" s="55"/>
     </row>
     <row r="3" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -8700,7 +8733,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="52" t="s">
+      <c r="M12" s="46" t="s">
         <v>709</v>
       </c>
       <c r="N12" s="2"/>
@@ -8728,7 +8761,7 @@
       <c r="Z12" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AA12" s="52" t="s">
+      <c r="AA12" s="46" t="s">
         <v>709</v>
       </c>
       <c r="AB12" s="2"/>
@@ -9110,7 +9143,7 @@
         <v>85</v>
       </c>
       <c r="AB18" s="2"/>
-      <c r="AC18" s="52"/>
+      <c r="AC18" s="46"/>
       <c r="AD18" s="2"/>
       <c r="AE18" s="2"/>
       <c r="AF18" s="2"/>
@@ -9154,7 +9187,7 @@
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-      <c r="P19" s="54" t="s">
+      <c r="P19" s="48" t="s">
         <v>710</v>
       </c>
       <c r="Q19" s="2"/>
@@ -9223,7 +9256,7 @@
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
-      <c r="P20" s="54" t="s">
+      <c r="P20" s="48" t="s">
         <v>711</v>
       </c>
       <c r="Q20" s="2"/>
@@ -9311,7 +9344,7 @@
         <v>80</v>
       </c>
       <c r="AB21" s="2"/>
-      <c r="AC21" s="52" t="s">
+      <c r="AC21" s="46" t="s">
         <v>714</v>
       </c>
       <c r="AD21" s="2"/>
@@ -11358,45 +11391,45 @@
       <c r="AK59" s="1"/>
     </row>
     <row r="60" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="45" t="s">
+      <c r="A60" s="53" t="s">
         <v>532</v>
       </c>
-      <c r="B60" s="46"/>
-      <c r="C60" s="46"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="46"/>
-      <c r="J60" s="46"/>
-      <c r="K60" s="46"/>
-      <c r="L60" s="46"/>
-      <c r="M60" s="46"/>
-      <c r="N60" s="46"/>
-      <c r="O60" s="46"/>
-      <c r="P60" s="46"/>
-      <c r="Q60" s="46"/>
-      <c r="R60" s="46"/>
-      <c r="S60" s="46"/>
-      <c r="T60" s="46"/>
-      <c r="U60" s="46"/>
-      <c r="V60" s="46"/>
-      <c r="W60" s="46"/>
-      <c r="X60" s="46"/>
-      <c r="Y60" s="46"/>
-      <c r="Z60" s="46"/>
-      <c r="AA60" s="46"/>
-      <c r="AB60" s="46"/>
-      <c r="AC60" s="46"/>
-      <c r="AD60" s="46"/>
-      <c r="AE60" s="46"/>
-      <c r="AF60" s="46"/>
-      <c r="AG60" s="46"/>
-      <c r="AH60" s="46"/>
-      <c r="AI60" s="46"/>
-      <c r="AJ60" s="46"/>
-      <c r="AK60" s="47"/>
+      <c r="B60" s="54"/>
+      <c r="C60" s="54"/>
+      <c r="D60" s="54"/>
+      <c r="E60" s="54"/>
+      <c r="F60" s="54"/>
+      <c r="G60" s="54"/>
+      <c r="H60" s="54"/>
+      <c r="I60" s="54"/>
+      <c r="J60" s="54"/>
+      <c r="K60" s="54"/>
+      <c r="L60" s="54"/>
+      <c r="M60" s="54"/>
+      <c r="N60" s="54"/>
+      <c r="O60" s="54"/>
+      <c r="P60" s="54"/>
+      <c r="Q60" s="54"/>
+      <c r="R60" s="54"/>
+      <c r="S60" s="54"/>
+      <c r="T60" s="54"/>
+      <c r="U60" s="54"/>
+      <c r="V60" s="54"/>
+      <c r="W60" s="54"/>
+      <c r="X60" s="54"/>
+      <c r="Y60" s="54"/>
+      <c r="Z60" s="54"/>
+      <c r="AA60" s="54"/>
+      <c r="AB60" s="54"/>
+      <c r="AC60" s="54"/>
+      <c r="AD60" s="54"/>
+      <c r="AE60" s="54"/>
+      <c r="AF60" s="54"/>
+      <c r="AG60" s="54"/>
+      <c r="AH60" s="54"/>
+      <c r="AI60" s="54"/>
+      <c r="AJ60" s="54"/>
+      <c r="AK60" s="55"/>
     </row>
     <row r="61" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
@@ -15201,45 +15234,45 @@
       <c r="AK128" s="1"/>
     </row>
     <row r="129" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="45" t="s">
+      <c r="A129" s="53" t="s">
         <v>531</v>
       </c>
-      <c r="B129" s="46"/>
-      <c r="C129" s="46"/>
-      <c r="D129" s="46"/>
-      <c r="E129" s="46"/>
-      <c r="F129" s="46"/>
-      <c r="G129" s="46"/>
-      <c r="H129" s="46"/>
-      <c r="I129" s="46"/>
-      <c r="J129" s="46"/>
-      <c r="K129" s="46"/>
-      <c r="L129" s="46"/>
-      <c r="M129" s="46"/>
-      <c r="N129" s="46"/>
-      <c r="O129" s="46"/>
-      <c r="P129" s="46"/>
-      <c r="Q129" s="46"/>
-      <c r="R129" s="46"/>
-      <c r="S129" s="46"/>
-      <c r="T129" s="46"/>
-      <c r="U129" s="46"/>
-      <c r="V129" s="46"/>
-      <c r="W129" s="46"/>
-      <c r="X129" s="46"/>
-      <c r="Y129" s="46"/>
-      <c r="Z129" s="46"/>
-      <c r="AA129" s="46"/>
-      <c r="AB129" s="46"/>
-      <c r="AC129" s="46"/>
-      <c r="AD129" s="46"/>
-      <c r="AE129" s="46"/>
-      <c r="AF129" s="46"/>
-      <c r="AG129" s="46"/>
-      <c r="AH129" s="46"/>
-      <c r="AI129" s="46"/>
-      <c r="AJ129" s="46"/>
-      <c r="AK129" s="47"/>
+      <c r="B129" s="54"/>
+      <c r="C129" s="54"/>
+      <c r="D129" s="54"/>
+      <c r="E129" s="54"/>
+      <c r="F129" s="54"/>
+      <c r="G129" s="54"/>
+      <c r="H129" s="54"/>
+      <c r="I129" s="54"/>
+      <c r="J129" s="54"/>
+      <c r="K129" s="54"/>
+      <c r="L129" s="54"/>
+      <c r="M129" s="54"/>
+      <c r="N129" s="54"/>
+      <c r="O129" s="54"/>
+      <c r="P129" s="54"/>
+      <c r="Q129" s="54"/>
+      <c r="R129" s="54"/>
+      <c r="S129" s="54"/>
+      <c r="T129" s="54"/>
+      <c r="U129" s="54"/>
+      <c r="V129" s="54"/>
+      <c r="W129" s="54"/>
+      <c r="X129" s="54"/>
+      <c r="Y129" s="54"/>
+      <c r="Z129" s="54"/>
+      <c r="AA129" s="54"/>
+      <c r="AB129" s="54"/>
+      <c r="AC129" s="54"/>
+      <c r="AD129" s="54"/>
+      <c r="AE129" s="54"/>
+      <c r="AF129" s="54"/>
+      <c r="AG129" s="54"/>
+      <c r="AH129" s="54"/>
+      <c r="AI129" s="54"/>
+      <c r="AJ129" s="54"/>
+      <c r="AK129" s="55"/>
     </row>
     <row r="130" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
@@ -15891,45 +15924,45 @@
       <c r="AK140" s="1"/>
     </row>
     <row r="141" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="45" t="s">
+      <c r="A141" s="53" t="s">
         <v>530</v>
       </c>
-      <c r="B141" s="46"/>
-      <c r="C141" s="46"/>
-      <c r="D141" s="46"/>
-      <c r="E141" s="46"/>
-      <c r="F141" s="46"/>
-      <c r="G141" s="46"/>
-      <c r="H141" s="46"/>
-      <c r="I141" s="46"/>
-      <c r="J141" s="46"/>
-      <c r="K141" s="46"/>
-      <c r="L141" s="46"/>
-      <c r="M141" s="46"/>
-      <c r="N141" s="46"/>
-      <c r="O141" s="46"/>
-      <c r="P141" s="46"/>
-      <c r="Q141" s="46"/>
-      <c r="R141" s="46"/>
-      <c r="S141" s="46"/>
-      <c r="T141" s="46"/>
-      <c r="U141" s="46"/>
-      <c r="V141" s="46"/>
-      <c r="W141" s="46"/>
-      <c r="X141" s="46"/>
-      <c r="Y141" s="46"/>
-      <c r="Z141" s="46"/>
-      <c r="AA141" s="46"/>
-      <c r="AB141" s="46"/>
-      <c r="AC141" s="46"/>
-      <c r="AD141" s="46"/>
-      <c r="AE141" s="46"/>
-      <c r="AF141" s="46"/>
-      <c r="AG141" s="46"/>
-      <c r="AH141" s="46"/>
-      <c r="AI141" s="46"/>
-      <c r="AJ141" s="46"/>
-      <c r="AK141" s="47"/>
+      <c r="B141" s="54"/>
+      <c r="C141" s="54"/>
+      <c r="D141" s="54"/>
+      <c r="E141" s="54"/>
+      <c r="F141" s="54"/>
+      <c r="G141" s="54"/>
+      <c r="H141" s="54"/>
+      <c r="I141" s="54"/>
+      <c r="J141" s="54"/>
+      <c r="K141" s="54"/>
+      <c r="L141" s="54"/>
+      <c r="M141" s="54"/>
+      <c r="N141" s="54"/>
+      <c r="O141" s="54"/>
+      <c r="P141" s="54"/>
+      <c r="Q141" s="54"/>
+      <c r="R141" s="54"/>
+      <c r="S141" s="54"/>
+      <c r="T141" s="54"/>
+      <c r="U141" s="54"/>
+      <c r="V141" s="54"/>
+      <c r="W141" s="54"/>
+      <c r="X141" s="54"/>
+      <c r="Y141" s="54"/>
+      <c r="Z141" s="54"/>
+      <c r="AA141" s="54"/>
+      <c r="AB141" s="54"/>
+      <c r="AC141" s="54"/>
+      <c r="AD141" s="54"/>
+      <c r="AE141" s="54"/>
+      <c r="AF141" s="54"/>
+      <c r="AG141" s="54"/>
+      <c r="AH141" s="54"/>
+      <c r="AI141" s="54"/>
+      <c r="AJ141" s="54"/>
+      <c r="AK141" s="55"/>
     </row>
     <row r="142" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
@@ -16485,7 +16518,7 @@
       <c r="J151" s="2"/>
       <c r="K151" s="2"/>
       <c r="L151" s="2"/>
-      <c r="M151" s="52" t="s">
+      <c r="M151" s="46" t="s">
         <v>709</v>
       </c>
       <c r="N151" s="2"/>
@@ -16505,7 +16538,7 @@
       <c r="Z151" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AA151" s="52" t="s">
+      <c r="AA151" s="46" t="s">
         <v>709</v>
       </c>
       <c r="AB151" s="2"/>
@@ -16756,7 +16789,7 @@
       </c>
       <c r="K156" s="2"/>
       <c r="L156" s="2"/>
-      <c r="M156" s="52" t="s">
+      <c r="M156" s="46" t="s">
         <v>707</v>
       </c>
       <c r="N156" s="2"/>
@@ -16773,7 +16806,7 @@
       <c r="Y156" s="2">
         <v>1</v>
       </c>
-      <c r="Z156" s="52" t="s">
+      <c r="Z156" s="46" t="s">
         <v>707</v>
       </c>
       <c r="AA156" s="2"/>
@@ -16813,7 +16846,7 @@
       </c>
       <c r="K157" s="2"/>
       <c r="L157" s="2"/>
-      <c r="M157" s="52" t="s">
+      <c r="M157" s="46" t="s">
         <v>133</v>
       </c>
       <c r="N157" s="2"/>
@@ -16846,45 +16879,45 @@
       <c r="AK157" s="2"/>
     </row>
     <row r="158" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="48" t="s">
+      <c r="A158" s="56" t="s">
         <v>529</v>
       </c>
-      <c r="B158" s="49"/>
-      <c r="C158" s="49"/>
-      <c r="D158" s="49"/>
-      <c r="E158" s="49"/>
-      <c r="F158" s="49"/>
-      <c r="G158" s="49"/>
-      <c r="H158" s="49"/>
-      <c r="I158" s="49"/>
-      <c r="J158" s="49"/>
-      <c r="K158" s="49"/>
-      <c r="L158" s="49"/>
-      <c r="M158" s="49"/>
-      <c r="N158" s="49"/>
-      <c r="O158" s="49"/>
-      <c r="P158" s="49"/>
-      <c r="Q158" s="49"/>
-      <c r="R158" s="49"/>
-      <c r="S158" s="49"/>
-      <c r="T158" s="49"/>
-      <c r="U158" s="49"/>
-      <c r="V158" s="49"/>
-      <c r="W158" s="49"/>
-      <c r="X158" s="49"/>
-      <c r="Y158" s="49"/>
-      <c r="Z158" s="49"/>
-      <c r="AA158" s="49"/>
-      <c r="AB158" s="49"/>
-      <c r="AC158" s="49"/>
-      <c r="AD158" s="49"/>
-      <c r="AE158" s="49"/>
-      <c r="AF158" s="49"/>
-      <c r="AG158" s="49"/>
-      <c r="AH158" s="49"/>
-      <c r="AI158" s="49"/>
-      <c r="AJ158" s="49"/>
-      <c r="AK158" s="50"/>
+      <c r="B158" s="57"/>
+      <c r="C158" s="57"/>
+      <c r="D158" s="57"/>
+      <c r="E158" s="57"/>
+      <c r="F158" s="57"/>
+      <c r="G158" s="57"/>
+      <c r="H158" s="57"/>
+      <c r="I158" s="57"/>
+      <c r="J158" s="57"/>
+      <c r="K158" s="57"/>
+      <c r="L158" s="57"/>
+      <c r="M158" s="57"/>
+      <c r="N158" s="57"/>
+      <c r="O158" s="57"/>
+      <c r="P158" s="57"/>
+      <c r="Q158" s="57"/>
+      <c r="R158" s="57"/>
+      <c r="S158" s="57"/>
+      <c r="T158" s="57"/>
+      <c r="U158" s="57"/>
+      <c r="V158" s="57"/>
+      <c r="W158" s="57"/>
+      <c r="X158" s="57"/>
+      <c r="Y158" s="57"/>
+      <c r="Z158" s="57"/>
+      <c r="AA158" s="57"/>
+      <c r="AB158" s="57"/>
+      <c r="AC158" s="57"/>
+      <c r="AD158" s="57"/>
+      <c r="AE158" s="57"/>
+      <c r="AF158" s="57"/>
+      <c r="AG158" s="57"/>
+      <c r="AH158" s="57"/>
+      <c r="AI158" s="57"/>
+      <c r="AJ158" s="57"/>
+      <c r="AK158" s="58"/>
     </row>
     <row r="159" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
@@ -17121,45 +17154,45 @@
       <c r="AK162" s="1"/>
     </row>
     <row r="163" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="45" t="s">
+      <c r="A163" s="53" t="s">
         <v>528</v>
       </c>
-      <c r="B163" s="46"/>
-      <c r="C163" s="46"/>
-      <c r="D163" s="46"/>
-      <c r="E163" s="46"/>
-      <c r="F163" s="46"/>
-      <c r="G163" s="46"/>
-      <c r="H163" s="46"/>
-      <c r="I163" s="46"/>
-      <c r="J163" s="46"/>
-      <c r="K163" s="46"/>
-      <c r="L163" s="46"/>
-      <c r="M163" s="46"/>
-      <c r="N163" s="46"/>
-      <c r="O163" s="46"/>
-      <c r="P163" s="46"/>
-      <c r="Q163" s="46"/>
-      <c r="R163" s="46"/>
-      <c r="S163" s="46"/>
-      <c r="T163" s="46"/>
-      <c r="U163" s="46"/>
-      <c r="V163" s="46"/>
-      <c r="W163" s="46"/>
-      <c r="X163" s="46"/>
-      <c r="Y163" s="46"/>
-      <c r="Z163" s="46"/>
-      <c r="AA163" s="46"/>
-      <c r="AB163" s="46"/>
-      <c r="AC163" s="46"/>
-      <c r="AD163" s="46"/>
-      <c r="AE163" s="46"/>
-      <c r="AF163" s="46"/>
-      <c r="AG163" s="46"/>
-      <c r="AH163" s="46"/>
-      <c r="AI163" s="46"/>
-      <c r="AJ163" s="46"/>
-      <c r="AK163" s="47"/>
+      <c r="B163" s="54"/>
+      <c r="C163" s="54"/>
+      <c r="D163" s="54"/>
+      <c r="E163" s="54"/>
+      <c r="F163" s="54"/>
+      <c r="G163" s="54"/>
+      <c r="H163" s="54"/>
+      <c r="I163" s="54"/>
+      <c r="J163" s="54"/>
+      <c r="K163" s="54"/>
+      <c r="L163" s="54"/>
+      <c r="M163" s="54"/>
+      <c r="N163" s="54"/>
+      <c r="O163" s="54"/>
+      <c r="P163" s="54"/>
+      <c r="Q163" s="54"/>
+      <c r="R163" s="54"/>
+      <c r="S163" s="54"/>
+      <c r="T163" s="54"/>
+      <c r="U163" s="54"/>
+      <c r="V163" s="54"/>
+      <c r="W163" s="54"/>
+      <c r="X163" s="54"/>
+      <c r="Y163" s="54"/>
+      <c r="Z163" s="54"/>
+      <c r="AA163" s="54"/>
+      <c r="AB163" s="54"/>
+      <c r="AC163" s="54"/>
+      <c r="AD163" s="54"/>
+      <c r="AE163" s="54"/>
+      <c r="AF163" s="54"/>
+      <c r="AG163" s="54"/>
+      <c r="AH163" s="54"/>
+      <c r="AI163" s="54"/>
+      <c r="AJ163" s="54"/>
+      <c r="AK163" s="55"/>
     </row>
     <row r="164" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
@@ -17451,45 +17484,45 @@
       <c r="AK168" s="1"/>
     </row>
     <row r="169" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A169" s="45" t="s">
+      <c r="A169" s="53" t="s">
         <v>527</v>
       </c>
-      <c r="B169" s="46"/>
-      <c r="C169" s="46"/>
-      <c r="D169" s="46"/>
-      <c r="E169" s="46"/>
-      <c r="F169" s="46"/>
-      <c r="G169" s="46"/>
-      <c r="H169" s="46"/>
-      <c r="I169" s="46"/>
-      <c r="J169" s="46"/>
-      <c r="K169" s="46"/>
-      <c r="L169" s="46"/>
-      <c r="M169" s="46"/>
-      <c r="N169" s="46"/>
-      <c r="O169" s="46"/>
-      <c r="P169" s="46"/>
-      <c r="Q169" s="46"/>
-      <c r="R169" s="46"/>
-      <c r="S169" s="46"/>
-      <c r="T169" s="46"/>
-      <c r="U169" s="46"/>
-      <c r="V169" s="46"/>
-      <c r="W169" s="46"/>
-      <c r="X169" s="46"/>
-      <c r="Y169" s="46"/>
-      <c r="Z169" s="46"/>
-      <c r="AA169" s="46"/>
-      <c r="AB169" s="46"/>
-      <c r="AC169" s="46"/>
-      <c r="AD169" s="46"/>
-      <c r="AE169" s="46"/>
-      <c r="AF169" s="46"/>
-      <c r="AG169" s="46"/>
-      <c r="AH169" s="46"/>
-      <c r="AI169" s="46"/>
-      <c r="AJ169" s="46"/>
-      <c r="AK169" s="47"/>
+      <c r="B169" s="54"/>
+      <c r="C169" s="54"/>
+      <c r="D169" s="54"/>
+      <c r="E169" s="54"/>
+      <c r="F169" s="54"/>
+      <c r="G169" s="54"/>
+      <c r="H169" s="54"/>
+      <c r="I169" s="54"/>
+      <c r="J169" s="54"/>
+      <c r="K169" s="54"/>
+      <c r="L169" s="54"/>
+      <c r="M169" s="54"/>
+      <c r="N169" s="54"/>
+      <c r="O169" s="54"/>
+      <c r="P169" s="54"/>
+      <c r="Q169" s="54"/>
+      <c r="R169" s="54"/>
+      <c r="S169" s="54"/>
+      <c r="T169" s="54"/>
+      <c r="U169" s="54"/>
+      <c r="V169" s="54"/>
+      <c r="W169" s="54"/>
+      <c r="X169" s="54"/>
+      <c r="Y169" s="54"/>
+      <c r="Z169" s="54"/>
+      <c r="AA169" s="54"/>
+      <c r="AB169" s="54"/>
+      <c r="AC169" s="54"/>
+      <c r="AD169" s="54"/>
+      <c r="AE169" s="54"/>
+      <c r="AF169" s="54"/>
+      <c r="AG169" s="54"/>
+      <c r="AH169" s="54"/>
+      <c r="AI169" s="54"/>
+      <c r="AJ169" s="54"/>
+      <c r="AK169" s="55"/>
     </row>
     <row r="170" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
@@ -17952,45 +17985,45 @@
       <c r="AK177" s="1"/>
     </row>
     <row r="178" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A178" s="45" t="s">
+      <c r="A178" s="53" t="s">
         <v>526</v>
       </c>
-      <c r="B178" s="46"/>
-      <c r="C178" s="46"/>
-      <c r="D178" s="46"/>
-      <c r="E178" s="46"/>
-      <c r="F178" s="46"/>
-      <c r="G178" s="46"/>
-      <c r="H178" s="46"/>
-      <c r="I178" s="46"/>
-      <c r="J178" s="46"/>
-      <c r="K178" s="46"/>
-      <c r="L178" s="46"/>
-      <c r="M178" s="46"/>
-      <c r="N178" s="46"/>
-      <c r="O178" s="46"/>
-      <c r="P178" s="46"/>
-      <c r="Q178" s="46"/>
-      <c r="R178" s="46"/>
-      <c r="S178" s="46"/>
-      <c r="T178" s="46"/>
-      <c r="U178" s="46"/>
-      <c r="V178" s="46"/>
-      <c r="W178" s="46"/>
-      <c r="X178" s="46"/>
-      <c r="Y178" s="46"/>
-      <c r="Z178" s="46"/>
-      <c r="AA178" s="46"/>
-      <c r="AB178" s="46"/>
-      <c r="AC178" s="46"/>
-      <c r="AD178" s="46"/>
-      <c r="AE178" s="46"/>
-      <c r="AF178" s="46"/>
-      <c r="AG178" s="46"/>
-      <c r="AH178" s="46"/>
-      <c r="AI178" s="46"/>
-      <c r="AJ178" s="46"/>
-      <c r="AK178" s="47"/>
+      <c r="B178" s="54"/>
+      <c r="C178" s="54"/>
+      <c r="D178" s="54"/>
+      <c r="E178" s="54"/>
+      <c r="F178" s="54"/>
+      <c r="G178" s="54"/>
+      <c r="H178" s="54"/>
+      <c r="I178" s="54"/>
+      <c r="J178" s="54"/>
+      <c r="K178" s="54"/>
+      <c r="L178" s="54"/>
+      <c r="M178" s="54"/>
+      <c r="N178" s="54"/>
+      <c r="O178" s="54"/>
+      <c r="P178" s="54"/>
+      <c r="Q178" s="54"/>
+      <c r="R178" s="54"/>
+      <c r="S178" s="54"/>
+      <c r="T178" s="54"/>
+      <c r="U178" s="54"/>
+      <c r="V178" s="54"/>
+      <c r="W178" s="54"/>
+      <c r="X178" s="54"/>
+      <c r="Y178" s="54"/>
+      <c r="Z178" s="54"/>
+      <c r="AA178" s="54"/>
+      <c r="AB178" s="54"/>
+      <c r="AC178" s="54"/>
+      <c r="AD178" s="54"/>
+      <c r="AE178" s="54"/>
+      <c r="AF178" s="54"/>
+      <c r="AG178" s="54"/>
+      <c r="AH178" s="54"/>
+      <c r="AI178" s="54"/>
+      <c r="AJ178" s="54"/>
+      <c r="AK178" s="55"/>
     </row>
     <row r="179" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A179" s="26" t="s">
@@ -18398,45 +18431,45 @@
       <c r="AK185" s="1"/>
     </row>
     <row r="186" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A186" s="45" t="s">
+      <c r="A186" s="53" t="s">
         <v>534</v>
       </c>
-      <c r="B186" s="46"/>
-      <c r="C186" s="46"/>
-      <c r="D186" s="46"/>
-      <c r="E186" s="46"/>
-      <c r="F186" s="46"/>
-      <c r="G186" s="46"/>
-      <c r="H186" s="46"/>
-      <c r="I186" s="46"/>
-      <c r="J186" s="46"/>
-      <c r="K186" s="46"/>
-      <c r="L186" s="46"/>
-      <c r="M186" s="46"/>
-      <c r="N186" s="46"/>
-      <c r="O186" s="46"/>
-      <c r="P186" s="46"/>
-      <c r="Q186" s="46"/>
-      <c r="R186" s="46"/>
-      <c r="S186" s="46"/>
-      <c r="T186" s="46"/>
-      <c r="U186" s="46"/>
-      <c r="V186" s="46"/>
-      <c r="W186" s="46"/>
-      <c r="X186" s="46"/>
-      <c r="Y186" s="46"/>
-      <c r="Z186" s="46"/>
-      <c r="AA186" s="46"/>
-      <c r="AB186" s="46"/>
-      <c r="AC186" s="46"/>
-      <c r="AD186" s="46"/>
-      <c r="AE186" s="46"/>
-      <c r="AF186" s="46"/>
-      <c r="AG186" s="46"/>
-      <c r="AH186" s="46"/>
-      <c r="AI186" s="46"/>
-      <c r="AJ186" s="46"/>
-      <c r="AK186" s="47"/>
+      <c r="B186" s="54"/>
+      <c r="C186" s="54"/>
+      <c r="D186" s="54"/>
+      <c r="E186" s="54"/>
+      <c r="F186" s="54"/>
+      <c r="G186" s="54"/>
+      <c r="H186" s="54"/>
+      <c r="I186" s="54"/>
+      <c r="J186" s="54"/>
+      <c r="K186" s="54"/>
+      <c r="L186" s="54"/>
+      <c r="M186" s="54"/>
+      <c r="N186" s="54"/>
+      <c r="O186" s="54"/>
+      <c r="P186" s="54"/>
+      <c r="Q186" s="54"/>
+      <c r="R186" s="54"/>
+      <c r="S186" s="54"/>
+      <c r="T186" s="54"/>
+      <c r="U186" s="54"/>
+      <c r="V186" s="54"/>
+      <c r="W186" s="54"/>
+      <c r="X186" s="54"/>
+      <c r="Y186" s="54"/>
+      <c r="Z186" s="54"/>
+      <c r="AA186" s="54"/>
+      <c r="AB186" s="54"/>
+      <c r="AC186" s="54"/>
+      <c r="AD186" s="54"/>
+      <c r="AE186" s="54"/>
+      <c r="AF186" s="54"/>
+      <c r="AG186" s="54"/>
+      <c r="AH186" s="54"/>
+      <c r="AI186" s="54"/>
+      <c r="AJ186" s="54"/>
+      <c r="AK186" s="55"/>
     </row>
     <row r="187" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
@@ -19213,45 +19246,45 @@
       <c r="AK200" s="2"/>
     </row>
     <row r="201" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A201" s="45" t="s">
+      <c r="A201" s="53" t="s">
         <v>535</v>
       </c>
-      <c r="B201" s="46"/>
-      <c r="C201" s="46"/>
-      <c r="D201" s="46"/>
-      <c r="E201" s="46"/>
-      <c r="F201" s="46"/>
-      <c r="G201" s="46"/>
-      <c r="H201" s="46"/>
-      <c r="I201" s="46"/>
-      <c r="J201" s="46"/>
-      <c r="K201" s="46"/>
-      <c r="L201" s="46"/>
-      <c r="M201" s="46"/>
-      <c r="N201" s="46"/>
-      <c r="O201" s="46"/>
-      <c r="P201" s="46"/>
-      <c r="Q201" s="46"/>
-      <c r="R201" s="46"/>
-      <c r="S201" s="46"/>
-      <c r="T201" s="46"/>
-      <c r="U201" s="46"/>
-      <c r="V201" s="46"/>
-      <c r="W201" s="46"/>
-      <c r="X201" s="46"/>
-      <c r="Y201" s="46"/>
-      <c r="Z201" s="46"/>
-      <c r="AA201" s="46"/>
-      <c r="AB201" s="46"/>
-      <c r="AC201" s="46"/>
-      <c r="AD201" s="46"/>
-      <c r="AE201" s="46"/>
-      <c r="AF201" s="46"/>
-      <c r="AG201" s="46"/>
-      <c r="AH201" s="46"/>
-      <c r="AI201" s="46"/>
-      <c r="AJ201" s="46"/>
-      <c r="AK201" s="47"/>
+      <c r="B201" s="54"/>
+      <c r="C201" s="54"/>
+      <c r="D201" s="54"/>
+      <c r="E201" s="54"/>
+      <c r="F201" s="54"/>
+      <c r="G201" s="54"/>
+      <c r="H201" s="54"/>
+      <c r="I201" s="54"/>
+      <c r="J201" s="54"/>
+      <c r="K201" s="54"/>
+      <c r="L201" s="54"/>
+      <c r="M201" s="54"/>
+      <c r="N201" s="54"/>
+      <c r="O201" s="54"/>
+      <c r="P201" s="54"/>
+      <c r="Q201" s="54"/>
+      <c r="R201" s="54"/>
+      <c r="S201" s="54"/>
+      <c r="T201" s="54"/>
+      <c r="U201" s="54"/>
+      <c r="V201" s="54"/>
+      <c r="W201" s="54"/>
+      <c r="X201" s="54"/>
+      <c r="Y201" s="54"/>
+      <c r="Z201" s="54"/>
+      <c r="AA201" s="54"/>
+      <c r="AB201" s="54"/>
+      <c r="AC201" s="54"/>
+      <c r="AD201" s="54"/>
+      <c r="AE201" s="54"/>
+      <c r="AF201" s="54"/>
+      <c r="AG201" s="54"/>
+      <c r="AH201" s="54"/>
+      <c r="AI201" s="54"/>
+      <c r="AJ201" s="54"/>
+      <c r="AK201" s="55"/>
     </row>
     <row r="202" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A202" s="1" t="s">
@@ -19586,45 +19619,45 @@
       <c r="AK207" s="1"/>
     </row>
     <row r="208" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A208" s="45" t="s">
+      <c r="A208" s="53" t="s">
         <v>549</v>
       </c>
-      <c r="B208" s="46"/>
-      <c r="C208" s="46"/>
-      <c r="D208" s="46"/>
-      <c r="E208" s="46"/>
-      <c r="F208" s="46"/>
-      <c r="G208" s="46"/>
-      <c r="H208" s="46"/>
-      <c r="I208" s="46"/>
-      <c r="J208" s="46"/>
-      <c r="K208" s="46"/>
-      <c r="L208" s="46"/>
-      <c r="M208" s="46"/>
-      <c r="N208" s="46"/>
-      <c r="O208" s="46"/>
-      <c r="P208" s="46"/>
-      <c r="Q208" s="46"/>
-      <c r="R208" s="46"/>
-      <c r="S208" s="46"/>
-      <c r="T208" s="46"/>
-      <c r="U208" s="46"/>
-      <c r="V208" s="46"/>
-      <c r="W208" s="46"/>
-      <c r="X208" s="46"/>
-      <c r="Y208" s="46"/>
-      <c r="Z208" s="46"/>
-      <c r="AA208" s="46"/>
-      <c r="AB208" s="46"/>
-      <c r="AC208" s="46"/>
-      <c r="AD208" s="46"/>
-      <c r="AE208" s="46"/>
-      <c r="AF208" s="46"/>
-      <c r="AG208" s="46"/>
-      <c r="AH208" s="46"/>
-      <c r="AI208" s="46"/>
-      <c r="AJ208" s="46"/>
-      <c r="AK208" s="47"/>
+      <c r="B208" s="54"/>
+      <c r="C208" s="54"/>
+      <c r="D208" s="54"/>
+      <c r="E208" s="54"/>
+      <c r="F208" s="54"/>
+      <c r="G208" s="54"/>
+      <c r="H208" s="54"/>
+      <c r="I208" s="54"/>
+      <c r="J208" s="54"/>
+      <c r="K208" s="54"/>
+      <c r="L208" s="54"/>
+      <c r="M208" s="54"/>
+      <c r="N208" s="54"/>
+      <c r="O208" s="54"/>
+      <c r="P208" s="54"/>
+      <c r="Q208" s="54"/>
+      <c r="R208" s="54"/>
+      <c r="S208" s="54"/>
+      <c r="T208" s="54"/>
+      <c r="U208" s="54"/>
+      <c r="V208" s="54"/>
+      <c r="W208" s="54"/>
+      <c r="X208" s="54"/>
+      <c r="Y208" s="54"/>
+      <c r="Z208" s="54"/>
+      <c r="AA208" s="54"/>
+      <c r="AB208" s="54"/>
+      <c r="AC208" s="54"/>
+      <c r="AD208" s="54"/>
+      <c r="AE208" s="54"/>
+      <c r="AF208" s="54"/>
+      <c r="AG208" s="54"/>
+      <c r="AH208" s="54"/>
+      <c r="AI208" s="54"/>
+      <c r="AJ208" s="54"/>
+      <c r="AK208" s="55"/>
     </row>
     <row r="209" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A209" s="1" t="s">
@@ -19963,45 +19996,45 @@
       <c r="AK214" s="1"/>
     </row>
     <row r="215" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="45" t="s">
+      <c r="A215" s="53" t="s">
         <v>740</v>
       </c>
-      <c r="B215" s="46"/>
-      <c r="C215" s="46"/>
-      <c r="D215" s="46"/>
-      <c r="E215" s="46"/>
-      <c r="F215" s="46"/>
-      <c r="G215" s="46"/>
-      <c r="H215" s="46"/>
-      <c r="I215" s="46"/>
-      <c r="J215" s="46"/>
-      <c r="K215" s="46"/>
-      <c r="L215" s="46"/>
-      <c r="M215" s="46"/>
-      <c r="N215" s="46"/>
-      <c r="O215" s="46"/>
-      <c r="P215" s="46"/>
-      <c r="Q215" s="46"/>
-      <c r="R215" s="46"/>
-      <c r="S215" s="46"/>
-      <c r="T215" s="46"/>
-      <c r="U215" s="46"/>
-      <c r="V215" s="46"/>
-      <c r="W215" s="46"/>
-      <c r="X215" s="46"/>
-      <c r="Y215" s="46"/>
-      <c r="Z215" s="46"/>
-      <c r="AA215" s="46"/>
-      <c r="AB215" s="46"/>
-      <c r="AC215" s="46"/>
-      <c r="AD215" s="46"/>
-      <c r="AE215" s="46"/>
-      <c r="AF215" s="46"/>
-      <c r="AG215" s="46"/>
-      <c r="AH215" s="46"/>
-      <c r="AI215" s="46"/>
-      <c r="AJ215" s="46"/>
-      <c r="AK215" s="47"/>
+      <c r="B215" s="54"/>
+      <c r="C215" s="54"/>
+      <c r="D215" s="54"/>
+      <c r="E215" s="54"/>
+      <c r="F215" s="54"/>
+      <c r="G215" s="54"/>
+      <c r="H215" s="54"/>
+      <c r="I215" s="54"/>
+      <c r="J215" s="54"/>
+      <c r="K215" s="54"/>
+      <c r="L215" s="54"/>
+      <c r="M215" s="54"/>
+      <c r="N215" s="54"/>
+      <c r="O215" s="54"/>
+      <c r="P215" s="54"/>
+      <c r="Q215" s="54"/>
+      <c r="R215" s="54"/>
+      <c r="S215" s="54"/>
+      <c r="T215" s="54"/>
+      <c r="U215" s="54"/>
+      <c r="V215" s="54"/>
+      <c r="W215" s="54"/>
+      <c r="X215" s="54"/>
+      <c r="Y215" s="54"/>
+      <c r="Z215" s="54"/>
+      <c r="AA215" s="54"/>
+      <c r="AB215" s="54"/>
+      <c r="AC215" s="54"/>
+      <c r="AD215" s="54"/>
+      <c r="AE215" s="54"/>
+      <c r="AF215" s="54"/>
+      <c r="AG215" s="54"/>
+      <c r="AH215" s="54"/>
+      <c r="AI215" s="54"/>
+      <c r="AJ215" s="54"/>
+      <c r="AK215" s="55"/>
     </row>
     <row r="216" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A216" s="1" t="s">
@@ -20611,45 +20644,45 @@
       <c r="AK226" s="1"/>
     </row>
     <row r="227" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A227" s="45" t="s">
+      <c r="A227" s="53" t="s">
         <v>741</v>
       </c>
-      <c r="B227" s="46"/>
-      <c r="C227" s="46"/>
-      <c r="D227" s="46"/>
-      <c r="E227" s="46"/>
-      <c r="F227" s="46"/>
-      <c r="G227" s="46"/>
-      <c r="H227" s="46"/>
-      <c r="I227" s="46"/>
-      <c r="J227" s="46"/>
-      <c r="K227" s="46"/>
-      <c r="L227" s="46"/>
-      <c r="M227" s="46"/>
-      <c r="N227" s="46"/>
-      <c r="O227" s="46"/>
-      <c r="P227" s="46"/>
-      <c r="Q227" s="46"/>
-      <c r="R227" s="46"/>
-      <c r="S227" s="46"/>
-      <c r="T227" s="46"/>
-      <c r="U227" s="46"/>
-      <c r="V227" s="46"/>
-      <c r="W227" s="46"/>
-      <c r="X227" s="46"/>
-      <c r="Y227" s="46"/>
-      <c r="Z227" s="46"/>
-      <c r="AA227" s="46"/>
-      <c r="AB227" s="46"/>
-      <c r="AC227" s="46"/>
-      <c r="AD227" s="46"/>
-      <c r="AE227" s="46"/>
-      <c r="AF227" s="46"/>
-      <c r="AG227" s="46"/>
-      <c r="AH227" s="46"/>
-      <c r="AI227" s="46"/>
-      <c r="AJ227" s="46"/>
-      <c r="AK227" s="47"/>
+      <c r="B227" s="54"/>
+      <c r="C227" s="54"/>
+      <c r="D227" s="54"/>
+      <c r="E227" s="54"/>
+      <c r="F227" s="54"/>
+      <c r="G227" s="54"/>
+      <c r="H227" s="54"/>
+      <c r="I227" s="54"/>
+      <c r="J227" s="54"/>
+      <c r="K227" s="54"/>
+      <c r="L227" s="54"/>
+      <c r="M227" s="54"/>
+      <c r="N227" s="54"/>
+      <c r="O227" s="54"/>
+      <c r="P227" s="54"/>
+      <c r="Q227" s="54"/>
+      <c r="R227" s="54"/>
+      <c r="S227" s="54"/>
+      <c r="T227" s="54"/>
+      <c r="U227" s="54"/>
+      <c r="V227" s="54"/>
+      <c r="W227" s="54"/>
+      <c r="X227" s="54"/>
+      <c r="Y227" s="54"/>
+      <c r="Z227" s="54"/>
+      <c r="AA227" s="54"/>
+      <c r="AB227" s="54"/>
+      <c r="AC227" s="54"/>
+      <c r="AD227" s="54"/>
+      <c r="AE227" s="54"/>
+      <c r="AF227" s="54"/>
+      <c r="AG227" s="54"/>
+      <c r="AH227" s="54"/>
+      <c r="AI227" s="54"/>
+      <c r="AJ227" s="54"/>
+      <c r="AK227" s="55"/>
     </row>
     <row r="228" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
@@ -20904,7 +20937,7 @@
       <c r="L232" s="1">
         <v>1</v>
       </c>
-      <c r="M232" s="53" t="s">
+      <c r="M232" s="47" t="s">
         <v>657</v>
       </c>
       <c r="N232" s="2"/>
@@ -21161,45 +21194,45 @@
       <c r="AK236" s="1"/>
     </row>
     <row r="237" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A237" s="45" t="s">
+      <c r="A237" s="53" t="s">
         <v>638</v>
       </c>
-      <c r="B237" s="46"/>
-      <c r="C237" s="46"/>
-      <c r="D237" s="46"/>
-      <c r="E237" s="46"/>
-      <c r="F237" s="46"/>
-      <c r="G237" s="46"/>
-      <c r="H237" s="46"/>
-      <c r="I237" s="46"/>
-      <c r="J237" s="46"/>
-      <c r="K237" s="46"/>
-      <c r="L237" s="46"/>
-      <c r="M237" s="46"/>
-      <c r="N237" s="46"/>
-      <c r="O237" s="46"/>
-      <c r="P237" s="46"/>
-      <c r="Q237" s="46"/>
-      <c r="R237" s="46"/>
-      <c r="S237" s="46"/>
-      <c r="T237" s="46"/>
-      <c r="U237" s="46"/>
-      <c r="V237" s="46"/>
-      <c r="W237" s="46"/>
-      <c r="X237" s="46"/>
-      <c r="Y237" s="46"/>
-      <c r="Z237" s="46"/>
-      <c r="AA237" s="46"/>
-      <c r="AB237" s="46"/>
-      <c r="AC237" s="46"/>
-      <c r="AD237" s="46"/>
-      <c r="AE237" s="46"/>
-      <c r="AF237" s="46"/>
-      <c r="AG237" s="46"/>
-      <c r="AH237" s="46"/>
-      <c r="AI237" s="46"/>
-      <c r="AJ237" s="46"/>
-      <c r="AK237" s="47"/>
+      <c r="B237" s="54"/>
+      <c r="C237" s="54"/>
+      <c r="D237" s="54"/>
+      <c r="E237" s="54"/>
+      <c r="F237" s="54"/>
+      <c r="G237" s="54"/>
+      <c r="H237" s="54"/>
+      <c r="I237" s="54"/>
+      <c r="J237" s="54"/>
+      <c r="K237" s="54"/>
+      <c r="L237" s="54"/>
+      <c r="M237" s="54"/>
+      <c r="N237" s="54"/>
+      <c r="O237" s="54"/>
+      <c r="P237" s="54"/>
+      <c r="Q237" s="54"/>
+      <c r="R237" s="54"/>
+      <c r="S237" s="54"/>
+      <c r="T237" s="54"/>
+      <c r="U237" s="54"/>
+      <c r="V237" s="54"/>
+      <c r="W237" s="54"/>
+      <c r="X237" s="54"/>
+      <c r="Y237" s="54"/>
+      <c r="Z237" s="54"/>
+      <c r="AA237" s="54"/>
+      <c r="AB237" s="54"/>
+      <c r="AC237" s="54"/>
+      <c r="AD237" s="54"/>
+      <c r="AE237" s="54"/>
+      <c r="AF237" s="54"/>
+      <c r="AG237" s="54"/>
+      <c r="AH237" s="54"/>
+      <c r="AI237" s="54"/>
+      <c r="AJ237" s="54"/>
+      <c r="AK237" s="55"/>
     </row>
     <row r="238" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A238" s="2" t="s">
@@ -21493,45 +21526,45 @@
       <c r="AK242" s="1"/>
     </row>
     <row r="243" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A243" s="45" t="s">
+      <c r="A243" s="53" t="s">
         <v>697</v>
       </c>
-      <c r="B243" s="46"/>
-      <c r="C243" s="46"/>
-      <c r="D243" s="46"/>
-      <c r="E243" s="46"/>
-      <c r="F243" s="46"/>
-      <c r="G243" s="46"/>
-      <c r="H243" s="46"/>
-      <c r="I243" s="46"/>
-      <c r="J243" s="46"/>
-      <c r="K243" s="46"/>
-      <c r="L243" s="46"/>
-      <c r="M243" s="46"/>
-      <c r="N243" s="46"/>
-      <c r="O243" s="46"/>
-      <c r="P243" s="46"/>
-      <c r="Q243" s="46"/>
-      <c r="R243" s="46"/>
-      <c r="S243" s="46"/>
-      <c r="T243" s="46"/>
-      <c r="U243" s="46"/>
-      <c r="V243" s="46"/>
-      <c r="W243" s="46"/>
-      <c r="X243" s="46"/>
-      <c r="Y243" s="46"/>
-      <c r="Z243" s="46"/>
-      <c r="AA243" s="46"/>
-      <c r="AB243" s="46"/>
-      <c r="AC243" s="46"/>
-      <c r="AD243" s="46"/>
-      <c r="AE243" s="46"/>
-      <c r="AF243" s="46"/>
-      <c r="AG243" s="46"/>
-      <c r="AH243" s="46"/>
-      <c r="AI243" s="46"/>
-      <c r="AJ243" s="46"/>
-      <c r="AK243" s="47"/>
+      <c r="B243" s="54"/>
+      <c r="C243" s="54"/>
+      <c r="D243" s="54"/>
+      <c r="E243" s="54"/>
+      <c r="F243" s="54"/>
+      <c r="G243" s="54"/>
+      <c r="H243" s="54"/>
+      <c r="I243" s="54"/>
+      <c r="J243" s="54"/>
+      <c r="K243" s="54"/>
+      <c r="L243" s="54"/>
+      <c r="M243" s="54"/>
+      <c r="N243" s="54"/>
+      <c r="O243" s="54"/>
+      <c r="P243" s="54"/>
+      <c r="Q243" s="54"/>
+      <c r="R243" s="54"/>
+      <c r="S243" s="54"/>
+      <c r="T243" s="54"/>
+      <c r="U243" s="54"/>
+      <c r="V243" s="54"/>
+      <c r="W243" s="54"/>
+      <c r="X243" s="54"/>
+      <c r="Y243" s="54"/>
+      <c r="Z243" s="54"/>
+      <c r="AA243" s="54"/>
+      <c r="AB243" s="54"/>
+      <c r="AC243" s="54"/>
+      <c r="AD243" s="54"/>
+      <c r="AE243" s="54"/>
+      <c r="AF243" s="54"/>
+      <c r="AG243" s="54"/>
+      <c r="AH243" s="54"/>
+      <c r="AI243" s="54"/>
+      <c r="AJ243" s="54"/>
+      <c r="AK243" s="55"/>
     </row>
     <row r="244" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A244" s="26" t="s">
@@ -21823,45 +21856,45 @@
       <c r="AK248" s="1"/>
     </row>
     <row r="249" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A249" s="45" t="s">
+      <c r="A249" s="53" t="s">
         <v>696</v>
       </c>
-      <c r="B249" s="46"/>
-      <c r="C249" s="46"/>
-      <c r="D249" s="46"/>
-      <c r="E249" s="46"/>
-      <c r="F249" s="46"/>
-      <c r="G249" s="46"/>
-      <c r="H249" s="46"/>
-      <c r="I249" s="46"/>
-      <c r="J249" s="46"/>
-      <c r="K249" s="46"/>
-      <c r="L249" s="46"/>
-      <c r="M249" s="46"/>
-      <c r="N249" s="46"/>
-      <c r="O249" s="46"/>
-      <c r="P249" s="46"/>
-      <c r="Q249" s="46"/>
-      <c r="R249" s="46"/>
-      <c r="S249" s="46"/>
-      <c r="T249" s="46"/>
-      <c r="U249" s="46"/>
-      <c r="V249" s="46"/>
-      <c r="W249" s="46"/>
-      <c r="X249" s="46"/>
-      <c r="Y249" s="46"/>
-      <c r="Z249" s="46"/>
-      <c r="AA249" s="46"/>
-      <c r="AB249" s="46"/>
-      <c r="AC249" s="46"/>
-      <c r="AD249" s="46"/>
-      <c r="AE249" s="46"/>
-      <c r="AF249" s="46"/>
-      <c r="AG249" s="46"/>
-      <c r="AH249" s="46"/>
-      <c r="AI249" s="46"/>
-      <c r="AJ249" s="46"/>
-      <c r="AK249" s="47"/>
+      <c r="B249" s="54"/>
+      <c r="C249" s="54"/>
+      <c r="D249" s="54"/>
+      <c r="E249" s="54"/>
+      <c r="F249" s="54"/>
+      <c r="G249" s="54"/>
+      <c r="H249" s="54"/>
+      <c r="I249" s="54"/>
+      <c r="J249" s="54"/>
+      <c r="K249" s="54"/>
+      <c r="L249" s="54"/>
+      <c r="M249" s="54"/>
+      <c r="N249" s="54"/>
+      <c r="O249" s="54"/>
+      <c r="P249" s="54"/>
+      <c r="Q249" s="54"/>
+      <c r="R249" s="54"/>
+      <c r="S249" s="54"/>
+      <c r="T249" s="54"/>
+      <c r="U249" s="54"/>
+      <c r="V249" s="54"/>
+      <c r="W249" s="54"/>
+      <c r="X249" s="54"/>
+      <c r="Y249" s="54"/>
+      <c r="Z249" s="54"/>
+      <c r="AA249" s="54"/>
+      <c r="AB249" s="54"/>
+      <c r="AC249" s="54"/>
+      <c r="AD249" s="54"/>
+      <c r="AE249" s="54"/>
+      <c r="AF249" s="54"/>
+      <c r="AG249" s="54"/>
+      <c r="AH249" s="54"/>
+      <c r="AI249" s="54"/>
+      <c r="AJ249" s="54"/>
+      <c r="AK249" s="55"/>
     </row>
     <row r="250" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A250" s="26" t="s">
@@ -22039,45 +22072,45 @@
       <c r="AK252" s="1"/>
     </row>
     <row r="253" spans="1:37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A253" s="45" t="s">
+      <c r="A253" s="53" t="s">
         <v>694</v>
       </c>
-      <c r="B253" s="46"/>
-      <c r="C253" s="46"/>
-      <c r="D253" s="46"/>
-      <c r="E253" s="46"/>
-      <c r="F253" s="46"/>
-      <c r="G253" s="46"/>
-      <c r="H253" s="46"/>
-      <c r="I253" s="46"/>
-      <c r="J253" s="46"/>
-      <c r="K253" s="46"/>
-      <c r="L253" s="46"/>
-      <c r="M253" s="46"/>
-      <c r="N253" s="46"/>
-      <c r="O253" s="46"/>
-      <c r="P253" s="46"/>
-      <c r="Q253" s="46"/>
-      <c r="R253" s="46"/>
-      <c r="S253" s="46"/>
-      <c r="T253" s="46"/>
-      <c r="U253" s="46"/>
-      <c r="V253" s="46"/>
-      <c r="W253" s="46"/>
-      <c r="X253" s="46"/>
-      <c r="Y253" s="46"/>
-      <c r="Z253" s="46"/>
-      <c r="AA253" s="46"/>
-      <c r="AB253" s="46"/>
-      <c r="AC253" s="46"/>
-      <c r="AD253" s="46"/>
-      <c r="AE253" s="46"/>
-      <c r="AF253" s="46"/>
-      <c r="AG253" s="46"/>
-      <c r="AH253" s="46"/>
-      <c r="AI253" s="46"/>
-      <c r="AJ253" s="46"/>
-      <c r="AK253" s="47"/>
+      <c r="B253" s="54"/>
+      <c r="C253" s="54"/>
+      <c r="D253" s="54"/>
+      <c r="E253" s="54"/>
+      <c r="F253" s="54"/>
+      <c r="G253" s="54"/>
+      <c r="H253" s="54"/>
+      <c r="I253" s="54"/>
+      <c r="J253" s="54"/>
+      <c r="K253" s="54"/>
+      <c r="L253" s="54"/>
+      <c r="M253" s="54"/>
+      <c r="N253" s="54"/>
+      <c r="O253" s="54"/>
+      <c r="P253" s="54"/>
+      <c r="Q253" s="54"/>
+      <c r="R253" s="54"/>
+      <c r="S253" s="54"/>
+      <c r="T253" s="54"/>
+      <c r="U253" s="54"/>
+      <c r="V253" s="54"/>
+      <c r="W253" s="54"/>
+      <c r="X253" s="54"/>
+      <c r="Y253" s="54"/>
+      <c r="Z253" s="54"/>
+      <c r="AA253" s="54"/>
+      <c r="AB253" s="54"/>
+      <c r="AC253" s="54"/>
+      <c r="AD253" s="54"/>
+      <c r="AE253" s="54"/>
+      <c r="AF253" s="54"/>
+      <c r="AG253" s="54"/>
+      <c r="AH253" s="54"/>
+      <c r="AI253" s="54"/>
+      <c r="AJ253" s="54"/>
+      <c r="AK253" s="55"/>
     </row>
     <row r="254" spans="1:37" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A254" s="2" t="s">
@@ -22237,6 +22270,14 @@
   </sheetData>
   <autoFilter ref="A1:AJ256" xr:uid="{0580B1DF-60C2-4E2B-940A-667729080FCF}"/>
   <mergeCells count="17">
+    <mergeCell ref="A169:AK169"/>
+    <mergeCell ref="A2:AK2"/>
+    <mergeCell ref="A60:AK60"/>
+    <mergeCell ref="A253:AK253"/>
+    <mergeCell ref="A249:AK249"/>
+    <mergeCell ref="A243:AK243"/>
+    <mergeCell ref="A237:AK237"/>
+    <mergeCell ref="A227:AK227"/>
     <mergeCell ref="A215:AK215"/>
     <mergeCell ref="A163:AK163"/>
     <mergeCell ref="A158:AK158"/>
@@ -22244,16 +22285,8 @@
     <mergeCell ref="A129:AK129"/>
     <mergeCell ref="A208:AK208"/>
     <mergeCell ref="A201:AK201"/>
-    <mergeCell ref="A253:AK253"/>
-    <mergeCell ref="A249:AK249"/>
-    <mergeCell ref="A243:AK243"/>
-    <mergeCell ref="A237:AK237"/>
-    <mergeCell ref="A227:AK227"/>
     <mergeCell ref="A186:AK186"/>
     <mergeCell ref="A178:AK178"/>
-    <mergeCell ref="A169:AK169"/>
-    <mergeCell ref="A2:AK2"/>
-    <mergeCell ref="A60:AK60"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22263,7 +22296,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC28CD21-0D0B-4F46-BC27-107466C7A67F}">
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr defaultColWidth="17.125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.25" style="32" customWidth="1"/>
@@ -22892,7 +22925,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="40"/>
-      <c r="J18" s="51" t="s">
+      <c r="J18" s="45" t="s">
         <v>641</v>
       </c>
       <c r="K18" s="29">
@@ -22931,7 +22964,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="29"/>
-      <c r="J19" s="51" t="s">
+      <c r="J19" s="45" t="s">
         <v>642</v>
       </c>
       <c r="K19" s="29">
@@ -23100,7 +23133,7 @@
         <v>1</v>
       </c>
       <c r="N23" s="29">
-        <v>1110</v>
+        <v>1200</v>
       </c>
       <c r="O23" s="29" t="s">
         <v>422</v>
@@ -23139,111 +23172,111 @@
         <v>1</v>
       </c>
       <c r="N24" s="29">
-        <v>1120</v>
+        <v>1300</v>
       </c>
       <c r="O24" s="30" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A25" s="29">
+    <row r="25" spans="1:15" ht="14.25" x14ac:dyDescent="0.3">
+      <c r="A25" s="50">
+        <v>1400</v>
+      </c>
+      <c r="B25" s="50">
+        <v>10</v>
+      </c>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50" t="s">
+        <v>744</v>
+      </c>
+      <c r="E25" s="50" t="s">
+        <v>745</v>
+      </c>
+      <c r="F25" s="50"/>
+      <c r="G25" s="51"/>
+      <c r="H25" s="50">
+        <v>0</v>
+      </c>
+      <c r="I25" s="51"/>
+      <c r="J25" s="52" t="s">
+        <v>743</v>
+      </c>
+      <c r="K25" s="50">
+        <v>1</v>
+      </c>
+      <c r="L25" s="50">
+        <v>0</v>
+      </c>
+      <c r="M25" s="50">
+        <v>1</v>
+      </c>
+      <c r="N25" s="50">
+        <v>1400</v>
+      </c>
+      <c r="O25" s="50" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="14.25" x14ac:dyDescent="0.3">
+      <c r="A26" s="50">
+        <v>1500</v>
+      </c>
+      <c r="B26" s="50">
+        <v>10</v>
+      </c>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50" t="s">
+        <v>746</v>
+      </c>
+      <c r="E26" s="50" t="s">
+        <v>747</v>
+      </c>
+      <c r="F26" s="50"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="50">
+        <v>0</v>
+      </c>
+      <c r="I26" s="51"/>
+      <c r="J26" s="52" t="s">
+        <v>743</v>
+      </c>
+      <c r="K26" s="50">
+        <v>1</v>
+      </c>
+      <c r="L26" s="50">
+        <v>0</v>
+      </c>
+      <c r="M26" s="50">
+        <v>1</v>
+      </c>
+      <c r="N26" s="50">
+        <v>1500</v>
+      </c>
+      <c r="O26" s="50" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A27" s="29">
         <v>30</v>
       </c>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29" t="s">
-        <v>414</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>415</v>
-      </c>
-      <c r="F25" s="29"/>
-      <c r="G25" s="40" t="s">
-        <v>298</v>
-      </c>
-      <c r="H25" s="29">
-        <v>0</v>
-      </c>
-      <c r="I25" s="29"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="29">
-        <v>1</v>
-      </c>
-      <c r="L25" s="29">
-        <v>0</v>
-      </c>
-      <c r="M25" s="30">
-        <v>1</v>
-      </c>
-      <c r="N25" s="29">
-        <v>91</v>
-      </c>
-      <c r="O25" s="29" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="14.25" x14ac:dyDescent="0.3">
-      <c r="A26" s="29">
-        <v>3010</v>
-      </c>
-      <c r="B26" s="29">
-        <v>30</v>
-      </c>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29" t="s">
-        <v>416</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>442</v>
-      </c>
-      <c r="F26" s="29"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="29">
-        <v>0</v>
-      </c>
-      <c r="I26" s="40"/>
-      <c r="J26" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="K26" s="29">
-        <v>1</v>
-      </c>
-      <c r="L26" s="29">
-        <v>0</v>
-      </c>
-      <c r="M26" s="30">
-        <v>1</v>
-      </c>
-      <c r="N26" s="29">
-        <v>9110</v>
-      </c>
-      <c r="O26" s="29" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="14.25" x14ac:dyDescent="0.3">
-      <c r="A27" s="29">
-        <v>3020</v>
-      </c>
-      <c r="B27" s="29">
-        <v>30</v>
-      </c>
+      <c r="B27" s="29"/>
       <c r="C27" s="29"/>
       <c r="D27" s="29" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>443</v>
+        <v>415</v>
       </c>
       <c r="F27" s="29"/>
-      <c r="G27" s="40"/>
+      <c r="G27" s="40" t="s">
+        <v>298</v>
+      </c>
       <c r="H27" s="29">
         <v>0</v>
       </c>
-      <c r="I27" s="40"/>
-      <c r="J27" s="7" t="s">
-        <v>419</v>
-      </c>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
       <c r="K27" s="29">
         <v>1</v>
       </c>
@@ -23254,25 +23287,25 @@
         <v>1</v>
       </c>
       <c r="N27" s="29">
-        <v>9120</v>
+        <v>91</v>
       </c>
       <c r="O27" s="29" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A28" s="29">
-        <v>3030</v>
+        <v>3010</v>
       </c>
       <c r="B28" s="29">
         <v>30</v>
       </c>
       <c r="C28" s="29"/>
       <c r="D28" s="29" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E28" s="29" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="F28" s="29"/>
       <c r="G28" s="40"/>
@@ -23280,8 +23313,8 @@
         <v>0</v>
       </c>
       <c r="I28" s="40"/>
-      <c r="J28" s="36" t="s">
-        <v>742</v>
+      <c r="J28" s="7" t="s">
+        <v>419</v>
       </c>
       <c r="K28" s="29">
         <v>1</v>
@@ -23293,9 +23326,87 @@
         <v>1</v>
       </c>
       <c r="N28" s="29">
+        <v>9110</v>
+      </c>
+      <c r="O28" s="29" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="14.25" x14ac:dyDescent="0.3">
+      <c r="A29" s="29">
+        <v>3020</v>
+      </c>
+      <c r="B29" s="29">
+        <v>30</v>
+      </c>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29" t="s">
+        <v>417</v>
+      </c>
+      <c r="E29" s="29" t="s">
+        <v>443</v>
+      </c>
+      <c r="F29" s="29"/>
+      <c r="G29" s="40"/>
+      <c r="H29" s="29">
+        <v>0</v>
+      </c>
+      <c r="I29" s="40"/>
+      <c r="J29" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="K29" s="29">
+        <v>1</v>
+      </c>
+      <c r="L29" s="29">
+        <v>0</v>
+      </c>
+      <c r="M29" s="30">
+        <v>1</v>
+      </c>
+      <c r="N29" s="29">
+        <v>9120</v>
+      </c>
+      <c r="O29" s="29" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A30" s="29">
+        <v>3030</v>
+      </c>
+      <c r="B30" s="29">
+        <v>30</v>
+      </c>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29" t="s">
+        <v>418</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>444</v>
+      </c>
+      <c r="F30" s="29"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="29">
+        <v>0</v>
+      </c>
+      <c r="I30" s="40"/>
+      <c r="J30" s="36" t="s">
+        <v>742</v>
+      </c>
+      <c r="K30" s="29">
+        <v>1</v>
+      </c>
+      <c r="L30" s="29">
+        <v>0</v>
+      </c>
+      <c r="M30" s="30">
+        <v>1</v>
+      </c>
+      <c r="N30" s="29">
         <v>9130</v>
       </c>
-      <c r="O28" s="29" t="s">
+      <c r="O30" s="29" t="s">
         <v>421</v>
       </c>
     </row>
@@ -23408,30 +23519,30 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="47" t="s">
         <v>644</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="47" t="s">
         <v>643</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53" t="s">
+      <c r="C2" s="47"/>
+      <c r="D2" s="47" t="s">
         <v>647</v>
       </c>
-      <c r="E2" s="53" t="s">
+      <c r="E2" s="47" t="s">
         <v>629</v>
       </c>
-      <c r="F2" s="53" t="s">
+      <c r="F2" s="47" t="s">
         <v>567</v>
       </c>
-      <c r="G2" s="53" t="s">
+      <c r="G2" s="47" t="s">
         <v>568</v>
       </c>
-      <c r="H2" s="53" t="s">
+      <c r="H2" s="47" t="s">
         <v>648</v>
       </c>
-      <c r="I2" s="55"/>
-      <c r="J2" s="53" t="s">
+      <c r="I2" s="49"/>
+      <c r="J2" s="47" t="s">
         <v>649</v>
       </c>
     </row>
@@ -23439,43 +23550,43 @@
       <c r="A3" s="2" t="s">
         <v>592</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="47" t="s">
         <v>656</v>
       </c>
-      <c r="C3" s="53"/>
+      <c r="C3" s="47"/>
       <c r="D3" s="26" t="s">
         <v>582</v>
       </c>
       <c r="E3" s="26" t="s">
         <v>655</v>
       </c>
-      <c r="F3" s="53" t="s">
+      <c r="F3" s="47" t="s">
         <v>568</v>
       </c>
-      <c r="G3" s="53" t="s">
+      <c r="G3" s="47" t="s">
         <v>567</v>
       </c>
-      <c r="H3" s="53"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="53" t="s">
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47" t="s">
         <v>654</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="47" t="s">
         <v>657</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
       <c r="D4" s="26"/>
       <c r="E4" s="26"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53" t="s">
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47" t="s">
         <v>659</v>
       </c>
-      <c r="J4" s="53" t="s">
+      <c r="J4" s="47" t="s">
         <v>658</v>
       </c>
     </row>

</xml_diff>